<commit_message>
Publish Prague_2024_WC, Vaires_2023_WC, Vaires_2024_OG
</commit_message>
<xml_diff>
--- a/events/Prague_2024_WC/Prague_2024_WC_start.xlsx
+++ b/events/Prague_2024_WC/Prague_2024_WC_start.xlsx
@@ -34067,12 +34067,12 @@
       </c>
       <c r="M532" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N532" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R532" t="inlineStr">
@@ -34145,12 +34145,12 @@
       </c>
       <c r="M533" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N533" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R533" t="inlineStr">
@@ -34223,12 +34223,12 @@
       </c>
       <c r="M534" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N534" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R534" t="inlineStr">
@@ -34301,12 +34301,12 @@
       </c>
       <c r="M535" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="N535" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R535" t="inlineStr">
@@ -34379,12 +34379,12 @@
       </c>
       <c r="M536" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="N536" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="R536" t="inlineStr">
@@ -34457,12 +34457,12 @@
       </c>
       <c r="M537" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="N537" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="R537" t="inlineStr">
@@ -34535,12 +34535,12 @@
       </c>
       <c r="M538" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N538" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="R538" t="inlineStr">
@@ -34613,12 +34613,12 @@
       </c>
       <c r="M539" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="N539" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="R539" t="inlineStr">

</xml_diff>